<commit_message>
Integrate CAR workflows and refine Fusion Studio workspace
</commit_message>
<xml_diff>
--- a/artifacts/framework-io/atlas.xlsx
+++ b/artifacts/framework-io/atlas.xlsx
@@ -195,7 +195,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>TTP Selection Studio</author>
+    <author>Fusion Studio</author>
   </authors>
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">
@@ -2009,7 +2009,7 @@
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>TTP Selection Studio</author>
+    <author>Fusion Studio</author>
   </authors>
   <commentList>
     <comment ref="A4" authorId="0" shapeId="0">

</xml_diff>